<commit_message>
Les mains.xlsx : derniere version (suppression de l'ancien nom de fichier)
</commit_message>
<xml_diff>
--- a/Les mains.xlsx
+++ b/Les mains.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanaismusic/Documents/CLIC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8732398-F7B9-FB4E-865F-9A2D2884660A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF263895-76C2-5748-B29A-6EC3FBDA3287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="40040" yWindow="2080" windowWidth="28040" windowHeight="17440" xr2:uid="{2F1647A4-8C84-E14B-83BA-CB692A19D8A6}"/>
   </bookViews>
@@ -1473,7 +1473,7 @@
         <v>86</v>
       </c>
       <c r="B87">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C87">
         <v>1</v>

</xml_diff>